<commit_message>
Live Proving Updated 19/10
</commit_message>
<xml_diff>
--- a/Wigan Transfer Note Data Extraction/Assets/IDP Config.xlsx
+++ b/Wigan Transfer Note Data Extraction/Assets/IDP Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://defra-my.sharepoint.com/personal/william_skalka_defra_gov_uk/Documents/Documents/GitHub/ea-wigan-waste-transfer-notes/Wigan Transfer Note Data Extraction/Assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="275" documentId="11_F25DC773A252ABDACC1048E8019B74A25BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D3152B6-0758-4CAB-A713-FF72944D578E}"/>
+  <xr:revisionPtr revIDLastSave="276" documentId="11_F25DC773A252ABDACC1048E8019B74A25BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA3A1A24-7F62-4F16-97AB-40A8F641933F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JDickinson" sheetId="1" r:id="rId1"/>
@@ -185,9 +185,6 @@
     <t>Registration Number (Section C)</t>
   </si>
   <si>
-    <t>Vehicle Registration (Section C)</t>
-  </si>
-  <si>
     <t>D1 Address of Transfer</t>
   </si>
   <si>
@@ -240,6 +237,9 @@
   </si>
   <si>
     <t>Receiving Site Authorisation</t>
+  </si>
+  <si>
+    <t>Details (Section C)</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1092,7 +1092,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1114,7 +1114,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -1125,7 +1125,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -1136,7 +1136,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -1147,7 +1147,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -1169,7 +1169,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B23">
         <v>1</v>
@@ -1206,7 +1206,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1217,7 +1217,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1228,7 +1228,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1239,7 +1239,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1250,7 +1250,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1261,7 +1261,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1272,7 +1272,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1294,7 +1294,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1305,7 +1305,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1316,7 +1316,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B12">
         <v>1</v>

</xml_diff>